<commit_message>
final working version 1
</commit_message>
<xml_diff>
--- a/data/extracted/extracted_questions.xlsx
+++ b/data/extracted/extracted_questions.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1304,6 +1304,2158 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>26433067858</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Select the option that is related to the third word in the same way as the second word
+is related to the first word. (The words must be considered as meaningful English
+words and must not be related to each other based on the number of letters/number of
+consonants/vowels in the word.)
+Animal : Zoology :: Plant : ?</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Geology</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>Palaeontology</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>Botany</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr"/>
+    </row>
+    <row r="18" ht="126" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>26433069255</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Which option represents the correct order of the given words as they would appear in
+the English dictionary?
+1 Sailboat
+2 Saint
+3 Sailor
+4 Sanction
+5 Sadly</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>3, 5, 1, 2, 4</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>5, 1, 3, 2, 4</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>5, 1, 3, 4, 2</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>5, 3, 1, 2, 4</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19" ht="162" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>26433093138</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Two Statements are given followed by Two conclusions numbered I and II. Assuming
+the statements to be true, even if they seem to be at variance with commonly known
+facts, decide which of the conclusions logically follow(s) from the statements.
+Statements:
+All buses are cars.
+No jeep is a car.
+Conclusions:
+I. No car is a jeep.
+II. No jeep is a bus.</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion II follows.</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>Neither conclusion I nor II follows.</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>Both conclusions I and II follows.</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I follows.</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>26433057903</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>In a code language, 'PARUL' is coded as RDTXN and 'MADHU' is coded as ODFKW.
+How will 'VIJAY' be coded in the same language?</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>XKLCB</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>XLLDA</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>XLMDA</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>XMLCA</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>26433085678</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Pointing at a girl, Seema said, “She is my father’s mother’s husband’s only son’s
+daughter.” How is that girl related to Seema?</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>Mother’s sister</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>Sister</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>Mother</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>Daughter</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="inlineStr"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>26433057314</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>In this question, the statement is followed by two conclusions. Which of the two
+conclusions is/are true?
+Statement: A ≤ D &lt; C = B &gt; E ≥ F &lt; G
+Conclusions: I. B &gt; A
+II. C &lt; F</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>Neither conclusion I nor II is true</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>Both conclusions I and II are true</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion II is true</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I is true</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>26433069199</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Which of the following numbers will replace the question mark (?) in the given series?
+3, 7, 5, 61, 363 ?</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>3367</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>3348</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>3630</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>3267</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr"/>
+    </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>26433068990</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Select the option that represents the letters that, when sequentially placed from left to
+right in the blanks below, will complete the letter series.
+_ M _ B A J M Q _ A _ M Q B _ J _ _ B _</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>J Q B J A M Q A</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>B Q A J M Q A B</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>A M B Q J M J Q</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>J A M M Q A B J</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr"/>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>26433079500</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>Town C is to the south of Town A. Town D is to the west of town A. Town B is to the
+east of town D. Town E is to the south of town B and south-east of Town C. What is the
+position of town A with respect to town B?</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>26433067321</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>In a certain code language, 'DAM’ is coded as '50' and 'PAD' is coded as '47'. How will
+'MAP' be coded in that language?</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr"/>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>26433056550</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Select the letter-cluster that will replace the question mark (?) in the given series and
+make it logically complete.
+FRP, HTR, JVT, ?, NZX</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>IWV</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>KWU</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>IUS</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>LXV</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="inlineStr"/>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>26433079440</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Which letter cluster will replace the question mark (?) to complete the given series?
+GROW, NJGG, ?, BTQA, ILIK</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>YDER</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>VIWQ</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>PSJW</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>UBYQ</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29" ht="126" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>26433069104</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>Select the set in which the number are related in the same way as the numbers of the
+given sets. (NOTE : Operations should be performed on the whole numbers, without
+breaking down the numbers into its constituent digits. E.g. 13 – Operations on 13 such
+as adding /subtracting /multiplying etc. to 13 can be performed. Breaking down 13 into
+1 and 3 and then performing mathematical operations on 1 and 3 is not allowed.)
+(182, 156, 13)
+(238, 212, 15)</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>(370, 348, 19)</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>(336, 302, 17)</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>(142, 126, 11)</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>(337, 311, 18)</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr"/>
+    </row>
+    <row r="30" ht="216" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>26433058075</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Read the given statements and conclusions carefully. Assuming that the information
+given in the statements is true, even if it appears to be at variance with commonly
+known facts, decide which of the given conclusions logically follow(s) from the
+statements.
+Statements:
+• All trojans are fairies.
+• No fairy is a flower.
+• All viruses are trojans.
+Conclusions:
+I. No flower is a trojan.
+II. Some viruses are trojans.
+III. No trojan is a virus.</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I follows</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I and III follow</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I and II follow</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion II follows</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr"/>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>26433067622</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Which of the following numbers will replace the question mark (?) in the given series?
+420, 462, 506, ?, 600, 650, 702</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>564</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>552</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>562</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>26433057236</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>Three of the following four letter-clusters are alike in a certain way and one is different.
+Pick the odd one out.</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>TWGD</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>ADZE</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="inlineStr">
+        <is>
+          <t>PSKH</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>FIUR</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33" ht="144" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>26433067918</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>Select the set in which the numbers are related in the same way as are the numbers of
+the following set.
+(NOTE: Operations should be performed on the whole numbers, without breaking
+down the numbers into its constituent digits. E.g. 13 – Operations on 13 such as
+adding /subtracting /multiplying etc. to 13 can be performed. Breaking down 13 into 1
+and 3 and then performing mathematical operations on 1 and 3 is NOT allowed)
+(212, 101, 111)
+(256, 123, 133)</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>(182, 74, 108)</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>(240, 105, 110)</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>(196, 89, 91)</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>(292, 122, 160)</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="inlineStr"/>
+    </row>
+    <row r="34" ht="54" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>26433068692</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>Select the correct combination of mathematical signs to sequentially replace the *
+signs and balance the given equation.
+65	*	56	*	8	*	19	*	2	*	34</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>−, ÷, −, ×, =</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>+, +, −, ×, =</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>+, ×, −, ×, =</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>+, ÷, −, ×, =</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>26433057998</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Three of the following four letter-clusters are alike in a certain way and one is different.
+Pick the odd one out.</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>MPJ</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>DIB</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>HKE</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>TWQ</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="inlineStr"/>
+    </row>
+    <row r="36" ht="216" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>26433058051</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Three statements are given followed by three conclusions numbered I, II and III.
+Assuming the statements to be true, even if they seem to be at variance with
+commonly known facts, decide which of the conclusions logically follow(s) from the
+statements.
+Statements:
+All beards are nails.
+Some nails are rings.
+All rings are pendants.
+Conclusions:
+I. All rings can never be nails.
+II. Some beards are rings.
+III. Some nails are pendants.</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusions II and III follow</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion III follows</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusions I and II follow</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusion I follows</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="inlineStr"/>
+    </row>
+    <row r="37" ht="126" customHeight="1">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>26433068349</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Select the set in which the numbers are NOT related in the same way as are the
+numbers of the given set.
+(NOTE: Operations should be performed on the whole numbers, without breaking
+down the numbers into its constituent digits. E.g. 13 – Operations on 13 such as
+adding /subtracting /multiplying etc. to 13 can be performed. Breaking down 13 into 1
+and 3 and then performing mathematical operations on 1 and 3 is not allowed)
+(16, 11, 377)</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>(12, 15, 367)</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>(16, 14, 452)</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>(14, 12, 340)</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>(18, 13, 493)</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="inlineStr"/>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>26433076698</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Town M is to the west of Town D. Town C is to the south-west of Town D. Town D is to
+the north of Town B. Town A is to the south of Town C. Town M is to the north of Town
+C. Town B is to the north-east of Town A.What is the position of Town B with respect to
+Town M?</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>South-east</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>North-west</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr"/>
+    </row>
+    <row r="39" ht="126" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>26433069113</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>Select the set in which the numbers are related in the same way as the numbers of the
+given sets. (NOTE : Operations should be performed on the whole numbers, without
+breaking down the numbers into its constituent digits. E.g. 13 – Operations on 13 such
+as adding /subtracting /multiplying etc. to 13 can be performed. Breaking down 13 into
+1 and 3 and then performing mathematical operations on 1 and 3 is not allowed.)
+(11, 100, 221)
+(14, 104, 300)</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>(15, 175, 390)</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>(17, 131, 410)</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>(19, 121, 445)</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>(13, 162, 331)</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr"/>
+    </row>
+    <row r="40" ht="54" customHeight="1">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>26433067684</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>Which two numbers from amongst the given options should be interchanged to make
+the given equation correct?
+(357 ÷ 2 + 3) ÷ 11 − 4 = (28 × 3 + 7) ÷ 9</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>11 and 28</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>2 and 3</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>7 and 9</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>2 and 9</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="inlineStr"/>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>26433067890</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Select the option that is related to the third number in the same way as the second
+number is related to the first number and the sixth number is related to the fifth
+number.
+6 : 43 :: 11 : ? :: 4 : 21</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="inlineStr"/>
+    </row>
+    <row r="42" ht="54" customHeight="1">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>26433057590</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Select the option that is related to the third term in the same way as the second term is
+related to the first term and the sixth term is related to the fifth term.
+16 : 50 :: 49 : ? :: 144 : 338</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43" ht="72" customHeight="1">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>26433056182</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>Select the option that is related to the fifth letter-cluster in the same way as the second
+letter-cluster is related to the first letter-cluster and the fourth letter-cluster is related
+to the third letter-cluster.
+MASTER : TSAMRE :: SMILES : LIMSSE :: FLIMSY : ?</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>FLIMYS</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>FILMYS</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>MILFYS</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>MLYFIS</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr"/>
+    </row>
+    <row r="44" ht="36" customHeight="1">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>26433067624</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>Which of the following numbers will replace the question mark (?) in the given series?
+144, 127, 110, ?, 76, 59</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr"/>
+    </row>
+    <row r="45" ht="72" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>26433091437</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>Six friends A, C, D, E, F and G are sitting in a straight row, facing north. They are
+waiting for their seventh friend B to join. Exactly three people are sitting to the left of
+A. C is occupying an end seat. F and D are immediate neighbours of G. If D is sitting to
+the immediate left of A, and E is second to the right of A, where will B sit?</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Fourth to the right of F</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Fifth to the right of G</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>To the immediate right of E</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>Third to the right of D</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="inlineStr"/>
+    </row>
+    <row r="46" ht="54" customHeight="1">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>26433067670</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>If A denotes ‘+’, B denotes ‘×’, C denotes ‘−’, and D denotes ‘÷’, then what will come in
+place of ‘?’ in the following equation?
+140 D 7 A 30 = 25 B ? D 8</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr"/>
+      <c r="J46" s="1" t="inlineStr"/>
+    </row>
+    <row r="47" ht="144" customHeight="1">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>26433068664</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Select the set in which the numbers are related in the same way as are the numbers of
+the following sets.
+(NOTE: Operations should be performed on the whole numbers, without breaking
+down the numbers into its constituent digits. E.g. 13 – Operations on 13 such as
+adding /subtracting /multiplying etc. to 13 can be performed. Breaking down 13 into 1
+and 3 and then performing mathematical operations on 1 and 3 is not allowed)
+(75, 55, 70)
+(65, 55, 68)</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>(95,	85,	124)</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>(95,	85,	104)</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>(95,	80,	104)</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>(90,	85,	104)</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr"/>
+    </row>
+    <row r="48" ht="36" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>26433067788</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>In a certain code language, 'FUTURE' is coded as ‘91’ and ‘MONEY’ is coded as ‘72’.
+How will 'SECURE' be coded in that language?</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="inlineStr"/>
+    </row>
+    <row r="49" ht="162" customHeight="1">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>26433087328</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>Study the given pattern carefully and select the number that can replace the question
+mark (?) in it.
+First row - 4, 6, 13
+Second row - 9, 8, 21
+Third row - 5, 6, ?
+(NOTE : Operations should be performed on the whole numbers, without breaking
+down the numbers into its constituent digits. Eg. 13 – Operations on 13 such as
+adding /deleting /multiplying etc. to 13 can be performed. Breaking down 13 into 1 and
+3 and then performing mathematical operations on 1 and 3 is not allowed)</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="inlineStr"/>
+    </row>
+    <row r="50" ht="36" customHeight="1">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>26433057905</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>In a code language, 'AMIT' is coded as 86 and 'VIJAY' is coded as</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>How will
+'GARIMA' be coded in the same language?</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr"/>
+    </row>
+    <row r="51" ht="54" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>26433067694</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>Which two symbols from amongst the given options should be interchanged to make
+the given equation correct?
+272 ÷ 17 − 196 ÷ ( 5 × 3 + 1) = 30</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>× and −</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>× and +</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>+ and ÷</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>+ and −</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr"/>
+    </row>
+    <row r="52" ht="216" customHeight="1">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>26433091627</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Three statements are given, followed by three conclusions numbered I, II and III.
+Assuming the statements to be true, even if they seem to be at variance with
+commonly known facts, decide which of the conclusions logically follow(s) from the
+statements.
+Statements:
+No toy is beautiful.
+Some beautiful are actresses.
+All actresses are rich.
+Conclusions:
+I. No toy is rich.
+II. Some actresses are beautiful.
+III. Some actresses are rich.</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusions II and III follow</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusions I and III follow</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>All the conclusions follow</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>Only conclusions I and II follow</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr"/>
+    </row>
+    <row r="53" ht="54" customHeight="1">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>26433067683</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>Which two symbols from amongst the given options should be interchanged to make
+the given equation correct?
+(35 – 2) × 3 = (56 × 8 ÷ 3 + 100) × 11</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>÷ and +</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>× and ÷</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>+ and −</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>× and −</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr"/>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>26433079386</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>Select the correct option that indicates the arrangement of the following words in a
+logical and meaningful order.</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>West Europe</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr"/>
+    </row>
+    <row r="55" ht="54" customHeight="1">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>26433069675</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>Select the correct combination of mathematical signs to replace the * signs and to
+balance the given equation.
+831 * 3 * 13 * 45 * 245 * 1</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>÷, +, −, =, ×</t>
+        </is>
+      </c>
+      <c r="G55" s="1">
+        <f>, ×, ÷, +, −</f>
+        <v/>
+      </c>
+      <c r="H55" s="1">
+        <f>, −, ÷, +, −</f>
+        <v/>
+      </c>
+      <c r="I55" s="1">
+        <f>, ÷, +, −, ×</f>
+        <v/>
+      </c>
+      <c r="J55" s="1" t="inlineStr"/>
+    </row>
+    <row r="56" ht="25" customHeight="1">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>26433093108</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>What will be the day of the week on 19th November 2053?</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="inlineStr"/>
+    </row>
+    <row r="57" ht="90" customHeight="1">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>26433086988</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>‘P + Q’ means ‘P is the daughter of Q’.
+‘P % Q’ means ‘P is the son of Q’.
+‘P # Q’ means ‘P is the wife of Q’.
+If A + B # C % D # E, which of the following statements is NOT correct?
+Section : General Awareness</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>C is the father of A.</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
+        <is>
+          <t>B is sister of E’s son.</t>
+        </is>
+      </c>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>D is the mother of B’s husband.</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>A is the daughter of E’s son.</t>
+        </is>
+      </c>
+      <c r="J57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58" ht="25" customHeight="1">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>SSC-Stenographer-Question-Paper-18-November-2022-Shift-1</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="inlineStr">
+        <is>
+          <t>26433085248</t>
+        </is>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>Who among the following Vijayanagara kings defeated the sultan of Bijapur in 1520?</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr">
+        <is>
+          <t>Deva Raya II</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
+        <is>
+          <t>Krishnadeva Raya</t>
+        </is>
+      </c>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>Vira Narasimha Raya</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>Bukka Raya I</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>